<commit_message>
feat: Implement new prediction pipeline with cached odds and injury data, and generate daily prediction reports.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-23.xlsx
+++ b/results/nba_predictions_2025-12-23.xlsx
@@ -568,10 +568,10 @@
         <v>53.33</v>
       </c>
       <c r="F2" t="n">
-        <v>57.82</v>
+        <v>57.85</v>
       </c>
       <c r="G2" t="n">
-        <v>42.18</v>
+        <v>42.15</v>
       </c>
       <c r="H2" t="n">
         <v>-0.77</v>
@@ -649,10 +649,10 @@
         <v>53.33</v>
       </c>
       <c r="F3" t="n">
-        <v>58.76</v>
+        <v>58.74</v>
       </c>
       <c r="G3" t="n">
-        <v>41.24</v>
+        <v>41.26</v>
       </c>
       <c r="H3" t="n">
         <v>-0.37</v>
@@ -734,10 +734,10 @@
         <v>60.61</v>
       </c>
       <c r="F4" t="n">
-        <v>57.12</v>
+        <v>57.15</v>
       </c>
       <c r="G4" t="n">
-        <v>42.88</v>
+        <v>42.85</v>
       </c>
       <c r="H4" t="n">
         <v>-0.19</v>
@@ -819,10 +819,10 @@
         <v>33.33</v>
       </c>
       <c r="F5" t="n">
-        <v>59.02</v>
+        <v>59.06</v>
       </c>
       <c r="G5" t="n">
-        <v>40.98</v>
+        <v>40.94</v>
       </c>
       <c r="H5" t="n">
         <v>0.09</v>
@@ -904,10 +904,10 @@
         <v>60.36</v>
       </c>
       <c r="F6" t="n">
-        <v>56.88</v>
+        <v>56.81</v>
       </c>
       <c r="G6" t="n">
-        <v>43.12</v>
+        <v>43.19</v>
       </c>
       <c r="H6" t="n">
         <v>-0.33</v>
@@ -989,10 +989,10 @@
         <v>53.33</v>
       </c>
       <c r="F7" t="n">
-        <v>59.07</v>
+        <v>59.22</v>
       </c>
       <c r="G7" t="n">
-        <v>40.93</v>
+        <v>40.78</v>
       </c>
       <c r="H7" t="n">
         <v>-0.11</v>
@@ -1070,10 +1070,10 @@
         <v>64.70999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>56.79</v>
+        <v>56.78</v>
       </c>
       <c r="G8" t="n">
-        <v>43.21</v>
+        <v>43.22</v>
       </c>
       <c r="H8" t="n">
         <v>-0.07000000000000001</v>
@@ -1118,8 +1118,16 @@
       <c r="T8" t="n">
         <v>26.6</v>
       </c>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Max Christie (DOUBTFUL)</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Tamar Bates (OUT)</t>
+        </is>
+      </c>
       <c r="W8" t="n">
         <v>-8.800000000000001</v>
       </c>
@@ -1147,10 +1155,10 @@
         <v>41.67</v>
       </c>
       <c r="F9" t="n">
-        <v>57.35</v>
+        <v>57.32</v>
       </c>
       <c r="G9" t="n">
-        <v>42.65</v>
+        <v>42.68</v>
       </c>
       <c r="H9" t="n">
         <v>-0.04</v>
@@ -1228,10 +1236,10 @@
         <v>53.33</v>
       </c>
       <c r="F10" t="n">
-        <v>54.2</v>
+        <v>54.28</v>
       </c>
       <c r="G10" t="n">
-        <v>45.8</v>
+        <v>45.72</v>
       </c>
       <c r="H10" t="n">
         <v>-0.05</v>
@@ -1281,7 +1289,11 @@
           <t>Harrison Ingram (OUT)</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Ousmane Dieng (OUT)</t>
+        </is>
+      </c>
       <c r="W10" t="n">
         <v>-2</v>
       </c>
@@ -1309,10 +1321,10 @@
         <v>53.33</v>
       </c>
       <c r="F11" t="n">
-        <v>56.56</v>
+        <v>56.76</v>
       </c>
       <c r="G11" t="n">
-        <v>43.44</v>
+        <v>43.24</v>
       </c>
       <c r="H11" t="n">
         <v>-0.35</v>
@@ -1394,10 +1406,10 @@
         <v>64.70999999999999</v>
       </c>
       <c r="F12" t="n">
-        <v>56.73</v>
+        <v>56.72</v>
       </c>
       <c r="G12" t="n">
-        <v>43.27</v>
+        <v>43.28</v>
       </c>
       <c r="H12" t="n">
         <v>-0.62</v>
@@ -1471,10 +1483,10 @@
         <v>60.61</v>
       </c>
       <c r="F13" t="n">
-        <v>57.52</v>
+        <v>57.51</v>
       </c>
       <c r="G13" t="n">
-        <v>42.48</v>
+        <v>42.49</v>
       </c>
       <c r="H13" t="n">
         <v>-0.28</v>
@@ -1548,10 +1560,10 @@
         <v>60.61</v>
       </c>
       <c r="F14" t="n">
-        <v>55.98</v>
+        <v>56.11</v>
       </c>
       <c r="G14" t="n">
-        <v>44.02</v>
+        <v>43.89</v>
       </c>
       <c r="H14" t="n">
         <v>-0.52</v>
@@ -1629,10 +1641,10 @@
         <v>53.33</v>
       </c>
       <c r="F15" t="n">
-        <v>54.2</v>
+        <v>54.18</v>
       </c>
       <c r="G15" t="n">
-        <v>45.8</v>
+        <v>45.82</v>
       </c>
       <c r="H15" t="n">
         <v>0.03</v>

</xml_diff>